<commit_message>
new updated the bug & improved the apis
</commit_message>
<xml_diff>
--- a/src/assets/formats/cinema/cinema/Cinema.xlsx
+++ b/src/assets/formats/cinema/cinema/Cinema.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5febf3aab2d16ef7/Desktop/New Proposals/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Backend plan generator\src\assets\formats\cinema\cinema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="13_ncr:1_{8B1A20C2-33F4-4597-968A-A05CF2A2C3EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84C192C7-C06F-4081-AD1B-B9AD69DCBAE4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{668C3626-0B03-43CB-BFF2-CEC1A15DC327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{B9EF980B-DC1D-4771-804F-15FCA6DD486A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{B9EF980B-DC1D-4771-804F-15FCA6DD486A}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="4" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t>Activity : 10 Sec A/V Format</t>
   </si>
@@ -106,15 +106,6 @@
   </si>
   <si>
     <t>Seating Capacity</t>
-  </si>
-  <si>
-    <t>Rates for 10 Sec :A/V Slide  (4 Weeks)</t>
-  </si>
-  <si>
-    <t>Total Screens : 58</t>
-  </si>
-  <si>
-    <t>Actual Cost : 4 Weeks</t>
   </si>
   <si>
     <t>Making &amp; Conversion Cost per Creative</t>
@@ -221,17 +212,41 @@
   <si>
     <t xml:space="preserve">The next evolution of adtech infrastructure and a unified command center that brings digital-level precision to every channel, both online and offline. Through a single, integrated dashboard, brands can plan, execute, and evaluate campaigns across all services, locations, and companies in one place, while gaining full transparency, real-time tracking, and performance visibility even for traditionally offline media. </t>
   </si>
+  <si>
+    <t xml:space="preserve">Total Screens : </t>
+  </si>
+  <si>
+    <t>Actual Cost :</t>
+  </si>
+  <si>
+    <t>Pincode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIER </t>
+  </si>
+  <si>
+    <t>Capacity Preference</t>
+  </si>
+  <si>
+    <t>Total Screen</t>
+  </si>
+  <si>
+    <t>Rates for 10 Sec :A/V Slide  (1 Week)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="8">
     <numFmt numFmtId="44" formatCode="_ &quot;₹&quot;\ * #,##0.00_ ;_ &quot;₹&quot;\ * \-#,##0.00_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="&quot;₹&quot;\ #,##0"/>
     <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="170" formatCode="_ &quot;₹&quot;\ * #,##0.00_ ;_ &quot;₹&quot;\ * \-#,##0.00_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="171" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="20" x14ac:knownFonts="1">
     <font>
@@ -333,20 +348,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="16"/>
       <color theme="0"/>
@@ -380,6 +381,22 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -407,7 +424,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -690,25 +707,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="5">
+  <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="170" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -752,6 +794,33 @@
     <xf numFmtId="0" fontId="11" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -791,15 +860,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -809,13 +869,46 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="3" borderId="18" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="3" borderId="23" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="3" borderId="7" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -827,73 +920,47 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="17" fillId="3" borderId="18" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="17" fillId="3" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="17" fillId="3" borderId="23" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="17" fillId="3" borderId="7" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="19" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="25" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="5">
+  <cellStyles count="9">
+    <cellStyle name="Comma 2" xfId="5" xr:uid="{3251317B-A39B-4BAB-9831-A3F2EEA27F73}"/>
     <cellStyle name="Comma 2 2" xfId="4" xr:uid="{CFDC4EF3-088C-4FAF-8B50-511F67987B0C}"/>
     <cellStyle name="Comma 3 3 2" xfId="2" xr:uid="{A9BF43A1-0478-414A-8CA7-3EBC41E3508A}"/>
+    <cellStyle name="Comma 3 3 2 2" xfId="7" xr:uid="{B15F4B50-F1F9-4CBF-9AEA-2C7556AD7E9D}"/>
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Currency 2" xfId="8" xr:uid="{F053EF0B-A51B-4121-8040-6D6627375023}"/>
     <cellStyle name="Currency 2 2" xfId="3" xr:uid="{78FF733A-69E9-40F9-BB13-13E42404AA02}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 10" xfId="6" xr:uid="{67859159-F889-4488-BDF7-45DB4BDD0186}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -923,10 +990,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>792480</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>751456</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>87630</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>2156</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -20629,8 +20696,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7509933" y="1062323"/>
-          <a:ext cx="6785187" cy="4441982"/>
+          <a:off x="7509933" y="1068673"/>
+          <a:ext cx="6785187" cy="4473732"/>
           <a:chOff x="7113693" y="1069943"/>
           <a:chExt cx="7105541" cy="4441982"/>
         </a:xfrm>
@@ -20751,8 +20818,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="152400" y="1059181"/>
-          <a:ext cx="7170420" cy="4450939"/>
+          <a:off x="152400" y="1065531"/>
+          <a:ext cx="7170420" cy="4482689"/>
           <a:chOff x="0" y="1066801"/>
           <a:chExt cx="7063740" cy="4450939"/>
         </a:xfrm>
@@ -21167,423 +21234,470 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{242F2B11-B48A-45E2-9B07-03817F7A4FD7}">
-  <dimension ref="A1:M23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:Q23"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="15.33203125" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.33203125" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" customWidth="1"/>
-    <col min="8" max="8" width="18.5546875" customWidth="1"/>
-    <col min="9" max="9" width="13.5546875" customWidth="1"/>
-    <col min="10" max="10" width="14.5546875" customWidth="1"/>
-    <col min="11" max="11" width="20" customWidth="1"/>
-    <col min="12" max="12" width="15.44140625" customWidth="1"/>
-    <col min="13" max="13" width="33.33203125" customWidth="1"/>
+    <col min="1" max="1" width="6.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.08984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19"/>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="20"/>
+    <row r="1" spans="1:17" ht="30.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="25"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="26"/>
     </row>
-    <row r="2" spans="1:13" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="19"/>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="20"/>
+    <row r="2" spans="1:17" ht="36.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="25"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="26"/>
     </row>
-    <row r="3" spans="1:13" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="19"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="20"/>
+    <row r="3" spans="1:17" ht="34.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="25"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="26"/>
     </row>
-    <row r="4" spans="1:13" ht="59.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="21"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="22"/>
+    <row r="4" spans="1:17" ht="59.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="27"/>
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+      <c r="M4" s="28"/>
     </row>
-    <row r="5" spans="1:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" cm="1">
+    <row r="5" spans="1:17" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="6" cm="1">
         <f t="array" aca="1" ref="A5" ca="1">A5:M7</f>
         <v>0</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="5" t="s">
+      <c r="B5" s="7"/>
+      <c r="C5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="10"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="24"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="29"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="29"/>
+      <c r="M5" s="30"/>
     </row>
-    <row r="6" spans="1:13" ht="11.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="11"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="7" t="s">
+    <row r="6" spans="1:17" ht="11.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="8"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
-      <c r="J6" s="25"/>
-      <c r="K6" s="25"/>
-      <c r="L6" s="25"/>
-      <c r="M6" s="26"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="31"/>
+      <c r="K6" s="31"/>
+      <c r="L6" s="31"/>
+      <c r="M6" s="32"/>
     </row>
-    <row r="7" spans="1:13" ht="9.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="12"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="27"/>
-      <c r="K7" s="27"/>
-      <c r="L7" s="27"/>
-      <c r="M7" s="28"/>
+    <row r="7" spans="1:17" ht="9.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="9"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="33"/>
+      <c r="J7" s="33"/>
+      <c r="K7" s="33"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="34"/>
     </row>
-    <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.3">
-      <c r="A8" s="32" t="s">
+    <row r="8" spans="1:17" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="58" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="33"/>
-      <c r="K8" s="33"/>
-      <c r="L8" s="33"/>
-      <c r="M8" s="34"/>
+      <c r="B8" s="59"/>
+      <c r="C8" s="59"/>
+      <c r="D8" s="59"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="59"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="59"/>
+      <c r="J8" s="59"/>
+      <c r="K8" s="59"/>
+      <c r="L8" s="59"/>
+      <c r="M8" s="59"/>
+      <c r="N8" s="59"/>
+      <c r="O8" s="59"/>
+      <c r="P8" s="59"/>
+      <c r="Q8" s="60"/>
     </row>
-    <row r="9" spans="1:13" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:17" ht="80.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="65" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="65" t="s">
         <v>8</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="I9" s="65" t="s">
         <v>10</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="J9" s="65" t="s">
+        <v>53</v>
+      </c>
+      <c r="K9" s="65" t="s">
+        <v>54</v>
+      </c>
+      <c r="L9" s="65" t="s">
+        <v>55</v>
+      </c>
+      <c r="M9" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="N9" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="O9" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="P9" s="65" t="s">
         <v>14</v>
       </c>
-      <c r="M9" s="3" t="s">
+      <c r="Q9" s="66" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="58.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="63"/>
+      <c r="B10" s="61"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="62"/>
+      <c r="H10" s="62"/>
+      <c r="I10" s="61"/>
+      <c r="J10" s="61"/>
+      <c r="K10" s="61"/>
+      <c r="L10" s="61"/>
+      <c r="M10" s="62"/>
+      <c r="N10" s="62"/>
+      <c r="O10" s="61"/>
+      <c r="P10" s="62"/>
+      <c r="Q10" s="67"/>
+    </row>
+    <row r="11" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="63"/>
+      <c r="B11" s="61"/>
+      <c r="C11" s="62"/>
+      <c r="D11" s="62"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="62"/>
+      <c r="H11" s="62"/>
+      <c r="I11" s="61"/>
+      <c r="J11" s="61"/>
+      <c r="K11" s="61"/>
+      <c r="L11" s="61"/>
+      <c r="M11" s="62"/>
+      <c r="N11" s="62"/>
+      <c r="O11" s="61"/>
+      <c r="P11" s="62"/>
+      <c r="Q11" s="67"/>
+    </row>
+    <row r="12" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="63"/>
+      <c r="B12" s="61"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="62"/>
+      <c r="H12" s="62"/>
+      <c r="I12" s="61"/>
+      <c r="J12" s="61"/>
+      <c r="K12" s="61"/>
+      <c r="L12" s="61"/>
+      <c r="M12" s="62"/>
+      <c r="N12" s="62"/>
+      <c r="O12" s="61"/>
+      <c r="P12" s="62"/>
+      <c r="Q12" s="67"/>
+    </row>
+    <row r="13" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="63"/>
+      <c r="B13" s="61"/>
+      <c r="C13" s="62"/>
+      <c r="D13" s="62"/>
+      <c r="E13" s="61"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="62"/>
+      <c r="H13" s="62"/>
+      <c r="I13" s="61"/>
+      <c r="J13" s="61"/>
+      <c r="K13" s="61"/>
+      <c r="L13" s="61"/>
+      <c r="M13" s="62"/>
+      <c r="N13" s="62"/>
+      <c r="O13" s="61"/>
+      <c r="P13" s="62"/>
+      <c r="Q13" s="67"/>
+    </row>
+    <row r="14" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="63"/>
+      <c r="B14" s="61"/>
+      <c r="C14" s="62"/>
+      <c r="D14" s="62"/>
+      <c r="E14" s="61"/>
+      <c r="F14" s="61"/>
+      <c r="G14" s="62"/>
+      <c r="H14" s="62"/>
+      <c r="I14" s="61"/>
+      <c r="J14" s="61"/>
+      <c r="K14" s="61"/>
+      <c r="L14" s="61"/>
+      <c r="M14" s="62"/>
+      <c r="N14" s="62"/>
+      <c r="O14" s="61"/>
+      <c r="P14" s="62"/>
+      <c r="Q14" s="67"/>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A15" s="63"/>
+      <c r="B15" s="61"/>
+      <c r="C15" s="62"/>
+      <c r="D15" s="62"/>
+      <c r="E15" s="61"/>
+      <c r="F15" s="61"/>
+      <c r="G15" s="62"/>
+      <c r="H15" s="62"/>
+      <c r="I15" s="61"/>
+      <c r="J15" s="61"/>
+      <c r="K15" s="61"/>
+      <c r="L15" s="61"/>
+      <c r="M15" s="62"/>
+      <c r="N15" s="62"/>
+      <c r="O15" s="61"/>
+      <c r="P15" s="62"/>
+      <c r="Q15" s="67"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A18" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="39"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="39"/>
+      <c r="G18" s="39"/>
+      <c r="H18" s="39"/>
+      <c r="I18" s="39"/>
+      <c r="J18" s="39"/>
+      <c r="K18" s="39"/>
+      <c r="L18" s="40"/>
+      <c r="M18" s="16"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A19" s="35" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="36"/>
+      <c r="I19" s="36"/>
+      <c r="J19" s="36"/>
+      <c r="K19" s="36"/>
+      <c r="L19" s="37"/>
+      <c r="M19" s="17"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A20" s="35" t="s">
         <v>15</v>
       </c>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="36"/>
+      <c r="I20" s="36"/>
+      <c r="J20" s="36"/>
+      <c r="K20" s="36"/>
+      <c r="L20" s="37"/>
+      <c r="M20" s="18"/>
     </row>
-    <row r="10" spans="1:13" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A18" s="35" t="s">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A21" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="36"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="36"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="36"/>
-      <c r="K18" s="36"/>
-      <c r="L18" s="37"/>
-      <c r="M18" s="54"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="36"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="36"/>
+      <c r="H21" s="36"/>
+      <c r="I21" s="36"/>
+      <c r="J21" s="36"/>
+      <c r="K21" s="36"/>
+      <c r="L21" s="37"/>
+      <c r="M21" s="19"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A19" s="29" t="s">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A22" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="30"/>
-      <c r="K19" s="30"/>
-      <c r="L19" s="31"/>
-      <c r="M19" s="55"/>
+      <c r="B22" s="36"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="36"/>
+      <c r="J22" s="36"/>
+      <c r="K22" s="36"/>
+      <c r="L22" s="37"/>
+      <c r="M22" s="19"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A20" s="29" t="s">
+    <row r="23" spans="1:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="30"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="30"/>
-      <c r="J20" s="30"/>
-      <c r="K20" s="30"/>
-      <c r="L20" s="31"/>
-      <c r="M20" s="56"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A21" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="30"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="30"/>
-      <c r="I21" s="30"/>
-      <c r="J21" s="30"/>
-      <c r="K21" s="30"/>
-      <c r="L21" s="31"/>
-      <c r="M21" s="57"/>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="30"/>
-      <c r="J22" s="30"/>
-      <c r="K22" s="30"/>
-      <c r="L22" s="31"/>
-      <c r="M22" s="57"/>
-    </row>
-    <row r="23" spans="1:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="18"/>
-      <c r="M23" s="58"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="14"/>
+      <c r="K23" s="14"/>
+      <c r="L23" s="15"/>
+      <c r="M23" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:M4"/>
     <mergeCell ref="E5:M7"/>
     <mergeCell ref="A22:L22"/>
-    <mergeCell ref="A8:M8"/>
     <mergeCell ref="A18:L18"/>
     <mergeCell ref="A19:L19"/>
     <mergeCell ref="A20:L20"/>
     <mergeCell ref="A21:L21"/>
+    <mergeCell ref="A8:Q8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -21593,404 +21707,414 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43B4FDE7-71EF-4EEB-ABD0-E0576A0C6A54}">
   <dimension ref="A1:N22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
-        <v>49</v>
+    <row r="1" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="44" t="s">
+        <v>46</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="51"/>
-      <c r="I1" s="51"/>
-      <c r="J1" s="51"/>
-      <c r="K1" s="51"/>
-      <c r="L1" s="51"/>
-      <c r="M1" s="51"/>
-      <c r="N1" s="51"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
     </row>
-    <row r="2" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="52"/>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-      <c r="I2" s="53"/>
-      <c r="J2" s="53"/>
-      <c r="K2" s="53"/>
-      <c r="L2" s="53"/>
-      <c r="M2" s="53"/>
-      <c r="N2" s="53"/>
+    <row r="2" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="46"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
+      <c r="N2" s="47"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="44" t="s">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A3" s="41" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42"/>
+      <c r="L3" s="42"/>
+      <c r="M3" s="42"/>
+      <c r="N3" s="43"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" s="41" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="42"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="42"/>
+      <c r="G4" s="42"/>
+      <c r="H4" s="42"/>
+      <c r="I4" s="42"/>
+      <c r="J4" s="42"/>
+      <c r="K4" s="42"/>
+      <c r="L4" s="42"/>
+      <c r="M4" s="42"/>
+      <c r="N4" s="43"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="42"/>
+      <c r="I5" s="42"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="42"/>
+      <c r="L5" s="42"/>
+      <c r="M5" s="42"/>
+      <c r="N5" s="43"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A6" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45"/>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
-      <c r="M3" s="45"/>
-      <c r="N3" s="46"/>
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="42"/>
+      <c r="F6" s="42"/>
+      <c r="G6" s="42"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="42"/>
+      <c r="K6" s="42"/>
+      <c r="L6" s="42"/>
+      <c r="M6" s="42"/>
+      <c r="N6" s="43"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="44" t="s">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
-      <c r="H4" s="45"/>
-      <c r="I4" s="45"/>
-      <c r="J4" s="45"/>
-      <c r="K4" s="45"/>
-      <c r="L4" s="45"/>
-      <c r="M4" s="45"/>
-      <c r="N4" s="46"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="42"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="42"/>
+      <c r="J7" s="42"/>
+      <c r="K7" s="42"/>
+      <c r="L7" s="42"/>
+      <c r="M7" s="42"/>
+      <c r="N7" s="43"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" s="44" t="s">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A8" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="45"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="45"/>
-      <c r="I5" s="45"/>
-      <c r="J5" s="45"/>
-      <c r="K5" s="45"/>
-      <c r="L5" s="45"/>
-      <c r="M5" s="45"/>
-      <c r="N5" s="46"/>
+      <c r="B8" s="42"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="42"/>
+      <c r="H8" s="42"/>
+      <c r="I8" s="42"/>
+      <c r="J8" s="42"/>
+      <c r="K8" s="42"/>
+      <c r="L8" s="42"/>
+      <c r="M8" s="42"/>
+      <c r="N8" s="43"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="44" t="s">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A9" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="45"/>
-      <c r="C6" s="45"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="45"/>
-      <c r="H6" s="45"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="45"/>
-      <c r="K6" s="45"/>
-      <c r="L6" s="45"/>
-      <c r="M6" s="45"/>
-      <c r="N6" s="46"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="42"/>
+      <c r="J9" s="42"/>
+      <c r="K9" s="42"/>
+      <c r="L9" s="42"/>
+      <c r="M9" s="42"/>
+      <c r="N9" s="43"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="44" t="s">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A10" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="45"/>
-      <c r="I7" s="45"/>
-      <c r="J7" s="45"/>
-      <c r="K7" s="45"/>
-      <c r="L7" s="45"/>
-      <c r="M7" s="45"/>
-      <c r="N7" s="46"/>
+      <c r="B10" s="42"/>
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
+      <c r="F10" s="42"/>
+      <c r="G10" s="42"/>
+      <c r="H10" s="42"/>
+      <c r="I10" s="42"/>
+      <c r="J10" s="42"/>
+      <c r="K10" s="42"/>
+      <c r="L10" s="42"/>
+      <c r="M10" s="42"/>
+      <c r="N10" s="43"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="44" t="s">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A11" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="45"/>
-      <c r="C8" s="45"/>
-      <c r="D8" s="45"/>
-      <c r="E8" s="45"/>
-      <c r="F8" s="45"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="45"/>
-      <c r="I8" s="45"/>
-      <c r="J8" s="45"/>
-      <c r="K8" s="45"/>
-      <c r="L8" s="45"/>
-      <c r="M8" s="45"/>
-      <c r="N8" s="46"/>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="42"/>
+      <c r="H11" s="42"/>
+      <c r="I11" s="42"/>
+      <c r="J11" s="42"/>
+      <c r="K11" s="42"/>
+      <c r="L11" s="42"/>
+      <c r="M11" s="42"/>
+      <c r="N11" s="43"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="44" t="s">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A12" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="45"/>
-      <c r="C9" s="45"/>
-      <c r="D9" s="45"/>
-      <c r="E9" s="45"/>
-      <c r="F9" s="45"/>
-      <c r="G9" s="45"/>
-      <c r="H9" s="45"/>
-      <c r="I9" s="45"/>
-      <c r="J9" s="45"/>
-      <c r="K9" s="45"/>
-      <c r="L9" s="45"/>
-      <c r="M9" s="45"/>
-      <c r="N9" s="46"/>
+      <c r="B12" s="42"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="42"/>
+      <c r="H12" s="42"/>
+      <c r="I12" s="42"/>
+      <c r="J12" s="42"/>
+      <c r="K12" s="42"/>
+      <c r="L12" s="42"/>
+      <c r="M12" s="42"/>
+      <c r="N12" s="43"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10" s="44" t="s">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A13" s="41" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="45"/>
-      <c r="C10" s="45"/>
-      <c r="D10" s="45"/>
-      <c r="E10" s="45"/>
-      <c r="F10" s="45"/>
-      <c r="G10" s="45"/>
-      <c r="H10" s="45"/>
-      <c r="I10" s="45"/>
-      <c r="J10" s="45"/>
-      <c r="K10" s="45"/>
-      <c r="L10" s="45"/>
-      <c r="M10" s="45"/>
-      <c r="N10" s="46"/>
+      <c r="B13" s="42"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="42"/>
+      <c r="F13" s="42"/>
+      <c r="G13" s="42"/>
+      <c r="H13" s="42"/>
+      <c r="I13" s="42"/>
+      <c r="J13" s="42"/>
+      <c r="K13" s="42"/>
+      <c r="L13" s="42"/>
+      <c r="M13" s="42"/>
+      <c r="N13" s="43"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="44" t="s">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A14" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="45"/>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="45"/>
-      <c r="F11" s="45"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="45"/>
-      <c r="I11" s="45"/>
-      <c r="J11" s="45"/>
-      <c r="K11" s="45"/>
-      <c r="L11" s="45"/>
-      <c r="M11" s="45"/>
-      <c r="N11" s="46"/>
+      <c r="B14" s="42"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="42"/>
+      <c r="H14" s="42"/>
+      <c r="I14" s="42"/>
+      <c r="J14" s="42"/>
+      <c r="K14" s="42"/>
+      <c r="L14" s="42"/>
+      <c r="M14" s="42"/>
+      <c r="N14" s="43"/>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="44" t="s">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A15" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="45"/>
-      <c r="C12" s="45"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="45"/>
-      <c r="F12" s="45"/>
-      <c r="G12" s="45"/>
-      <c r="H12" s="45"/>
-      <c r="I12" s="45"/>
-      <c r="J12" s="45"/>
-      <c r="K12" s="45"/>
-      <c r="L12" s="45"/>
-      <c r="M12" s="45"/>
-      <c r="N12" s="46"/>
+      <c r="B15" s="42"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="42"/>
+      <c r="F15" s="42"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="42"/>
+      <c r="J15" s="42"/>
+      <c r="K15" s="42"/>
+      <c r="L15" s="42"/>
+      <c r="M15" s="42"/>
+      <c r="N15" s="43"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="44" t="s">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A16" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="45"/>
-      <c r="C13" s="45"/>
-      <c r="D13" s="45"/>
-      <c r="E13" s="45"/>
-      <c r="F13" s="45"/>
-      <c r="G13" s="45"/>
-      <c r="H13" s="45"/>
-      <c r="I13" s="45"/>
-      <c r="J13" s="45"/>
-      <c r="K13" s="45"/>
-      <c r="L13" s="45"/>
-      <c r="M13" s="45"/>
-      <c r="N13" s="46"/>
+      <c r="B16" s="42"/>
+      <c r="C16" s="42"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="42"/>
+      <c r="F16" s="42"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="42"/>
+      <c r="I16" s="42"/>
+      <c r="J16" s="42"/>
+      <c r="K16" s="42"/>
+      <c r="L16" s="42"/>
+      <c r="M16" s="42"/>
+      <c r="N16" s="43"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" s="44" t="s">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A17" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="45"/>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="45"/>
-      <c r="I14" s="45"/>
-      <c r="J14" s="45"/>
-      <c r="K14" s="45"/>
-      <c r="L14" s="45"/>
-      <c r="M14" s="45"/>
-      <c r="N14" s="46"/>
+      <c r="B17" s="42"/>
+      <c r="C17" s="42"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="42"/>
+      <c r="F17" s="42"/>
+      <c r="G17" s="42"/>
+      <c r="H17" s="42"/>
+      <c r="I17" s="42"/>
+      <c r="J17" s="42"/>
+      <c r="K17" s="42"/>
+      <c r="L17" s="42"/>
+      <c r="M17" s="42"/>
+      <c r="N17" s="43"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="44" t="s">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A18" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="45"/>
-      <c r="C15" s="45"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="45"/>
-      <c r="F15" s="45"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="45"/>
-      <c r="I15" s="45"/>
-      <c r="J15" s="45"/>
-      <c r="K15" s="45"/>
-      <c r="L15" s="45"/>
-      <c r="M15" s="45"/>
-      <c r="N15" s="46"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="42"/>
+      <c r="D18" s="42"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="42"/>
+      <c r="H18" s="42"/>
+      <c r="I18" s="42"/>
+      <c r="J18" s="42"/>
+      <c r="K18" s="42"/>
+      <c r="L18" s="42"/>
+      <c r="M18" s="42"/>
+      <c r="N18" s="43"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="44" t="s">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A19" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="45"/>
-      <c r="C16" s="45"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="45"/>
-      <c r="F16" s="45"/>
-      <c r="G16" s="45"/>
-      <c r="H16" s="45"/>
-      <c r="I16" s="45"/>
-      <c r="J16" s="45"/>
-      <c r="K16" s="45"/>
-      <c r="L16" s="45"/>
-      <c r="M16" s="45"/>
-      <c r="N16" s="46"/>
+      <c r="B19" s="42"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="42"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="42"/>
+      <c r="H19" s="42"/>
+      <c r="I19" s="42"/>
+      <c r="J19" s="42"/>
+      <c r="K19" s="42"/>
+      <c r="L19" s="42"/>
+      <c r="M19" s="42"/>
+      <c r="N19" s="43"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="44" t="s">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A20" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="45"/>
-      <c r="C17" s="45"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="45"/>
-      <c r="F17" s="45"/>
-      <c r="G17" s="45"/>
-      <c r="H17" s="45"/>
-      <c r="I17" s="45"/>
-      <c r="J17" s="45"/>
-      <c r="K17" s="45"/>
-      <c r="L17" s="45"/>
-      <c r="M17" s="45"/>
-      <c r="N17" s="46"/>
+      <c r="B20" s="42"/>
+      <c r="C20" s="42"/>
+      <c r="D20" s="42"/>
+      <c r="E20" s="42"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="42"/>
+      <c r="H20" s="42"/>
+      <c r="I20" s="42"/>
+      <c r="J20" s="42"/>
+      <c r="K20" s="42"/>
+      <c r="L20" s="42"/>
+      <c r="M20" s="42"/>
+      <c r="N20" s="43"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="44" t="s">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A21" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="45"/>
-      <c r="C18" s="45"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="45"/>
-      <c r="G18" s="45"/>
-      <c r="H18" s="45"/>
-      <c r="I18" s="45"/>
-      <c r="J18" s="45"/>
-      <c r="K18" s="45"/>
-      <c r="L18" s="45"/>
-      <c r="M18" s="45"/>
-      <c r="N18" s="46"/>
+      <c r="B21" s="42"/>
+      <c r="C21" s="42"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="42"/>
+      <c r="G21" s="42"/>
+      <c r="H21" s="42"/>
+      <c r="I21" s="42"/>
+      <c r="J21" s="42"/>
+      <c r="K21" s="42"/>
+      <c r="L21" s="42"/>
+      <c r="M21" s="42"/>
+      <c r="N21" s="43"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="44" t="s">
+    <row r="22" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="45"/>
-      <c r="C19" s="45"/>
-      <c r="D19" s="45"/>
-      <c r="E19" s="45"/>
-      <c r="F19" s="45"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="45"/>
-      <c r="I19" s="45"/>
-      <c r="J19" s="45"/>
-      <c r="K19" s="45"/>
-      <c r="L19" s="45"/>
-      <c r="M19" s="45"/>
-      <c r="N19" s="46"/>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="44" t="s">
-        <v>39</v>
-      </c>
-      <c r="B20" s="45"/>
-      <c r="C20" s="45"/>
-      <c r="D20" s="45"/>
-      <c r="E20" s="45"/>
-      <c r="F20" s="45"/>
-      <c r="G20" s="45"/>
-      <c r="H20" s="45"/>
-      <c r="I20" s="45"/>
-      <c r="J20" s="45"/>
-      <c r="K20" s="45"/>
-      <c r="L20" s="45"/>
-      <c r="M20" s="45"/>
-      <c r="N20" s="46"/>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="44" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" s="45"/>
-      <c r="C21" s="45"/>
-      <c r="D21" s="45"/>
-      <c r="E21" s="45"/>
-      <c r="F21" s="45"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="45"/>
-      <c r="I21" s="45"/>
-      <c r="J21" s="45"/>
-      <c r="K21" s="45"/>
-      <c r="L21" s="45"/>
-      <c r="M21" s="45"/>
-      <c r="N21" s="46"/>
-    </row>
-    <row r="22" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="47" t="s">
-        <v>41</v>
-      </c>
-      <c r="B22" s="48"/>
-      <c r="C22" s="48"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="48"/>
-      <c r="F22" s="48"/>
-      <c r="G22" s="48"/>
-      <c r="H22" s="48"/>
-      <c r="I22" s="48"/>
-      <c r="J22" s="48"/>
-      <c r="K22" s="48"/>
-      <c r="L22" s="48"/>
-      <c r="M22" s="48"/>
-      <c r="N22" s="49"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="49"/>
+      <c r="I22" s="49"/>
+      <c r="J22" s="49"/>
+      <c r="K22" s="49"/>
+      <c r="L22" s="49"/>
+      <c r="M22" s="49"/>
+      <c r="N22" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A21:N21"/>
+    <mergeCell ref="A22:N22"/>
+    <mergeCell ref="A13:N13"/>
+    <mergeCell ref="A14:N14"/>
+    <mergeCell ref="A15:N15"/>
+    <mergeCell ref="A16:N16"/>
+    <mergeCell ref="A17:N17"/>
+    <mergeCell ref="A18:N18"/>
+    <mergeCell ref="A19:N19"/>
+    <mergeCell ref="A20:N20"/>
     <mergeCell ref="A12:N12"/>
     <mergeCell ref="A10:N10"/>
     <mergeCell ref="A3:N3"/>
@@ -22002,16 +22126,6 @@
     <mergeCell ref="A7:N7"/>
     <mergeCell ref="A8:N8"/>
     <mergeCell ref="A9:N9"/>
-    <mergeCell ref="A21:N21"/>
-    <mergeCell ref="A22:N22"/>
-    <mergeCell ref="A13:N13"/>
-    <mergeCell ref="A14:N14"/>
-    <mergeCell ref="A15:N15"/>
-    <mergeCell ref="A16:N16"/>
-    <mergeCell ref="A17:N17"/>
-    <mergeCell ref="A18:N18"/>
-    <mergeCell ref="A19:N19"/>
-    <mergeCell ref="A20:N20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -22021,485 +22135,485 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6825D90-E2AE-4788-8198-514C2F4DCC37}">
   <dimension ref="B1:M35"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="2:13" ht="21" x14ac:dyDescent="0.3">
-      <c r="B1" s="39" t="s">
+    <row r="1" spans="2:13" ht="21" x14ac:dyDescent="0.35">
+      <c r="B1" s="53" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="54"/>
+      <c r="J1" s="54"/>
+      <c r="K1" s="54"/>
+      <c r="L1" s="54"/>
+      <c r="M1" s="54"/>
+    </row>
+    <row r="2" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B2" s="55" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
+      <c r="M2" s="56"/>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="56"/>
+      <c r="I3" s="56"/>
+      <c r="J3" s="56"/>
+      <c r="K3" s="56"/>
+      <c r="L3" s="56"/>
+      <c r="M3" s="56"/>
+    </row>
+    <row r="4" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
+      <c r="K4" s="56"/>
+      <c r="L4" s="56"/>
+      <c r="M4" s="56"/>
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B5" s="55" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
+      <c r="C5" s="55"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="55"/>
+      <c r="G5" s="55"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="56"/>
+      <c r="K5" s="56"/>
+      <c r="L5" s="56"/>
+      <c r="M5" s="56"/>
     </row>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B2" s="41" t="s">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B6" s="57"/>
+      <c r="C6" s="57"/>
+      <c r="D6" s="57"/>
+      <c r="E6" s="57"/>
+      <c r="F6" s="57"/>
+      <c r="G6" s="57"/>
+      <c r="H6" s="56"/>
+      <c r="I6" s="56"/>
+      <c r="J6" s="56"/>
+      <c r="K6" s="56"/>
+      <c r="L6" s="56"/>
+      <c r="M6" s="56"/>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B7" s="57"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="57"/>
+      <c r="E7" s="57"/>
+      <c r="F7" s="57"/>
+      <c r="G7" s="57"/>
+      <c r="H7" s="56"/>
+      <c r="I7" s="56"/>
+      <c r="J7" s="56"/>
+      <c r="K7" s="56"/>
+      <c r="L7" s="56"/>
+      <c r="M7" s="56"/>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B8" s="55" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="42" t="s">
+      <c r="C8" s="55"/>
+      <c r="D8" s="55"/>
+      <c r="E8" s="55"/>
+      <c r="F8" s="55"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="56"/>
+      <c r="I8" s="56"/>
+      <c r="J8" s="56"/>
+      <c r="K8" s="56"/>
+      <c r="L8" s="56"/>
+      <c r="M8" s="56"/>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B9" s="57"/>
+      <c r="C9" s="57"/>
+      <c r="D9" s="57"/>
+      <c r="E9" s="57"/>
+      <c r="F9" s="57"/>
+      <c r="G9" s="57"/>
+      <c r="H9" s="56"/>
+      <c r="I9" s="56"/>
+      <c r="J9" s="56"/>
+      <c r="K9" s="56"/>
+      <c r="L9" s="56"/>
+      <c r="M9" s="56"/>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B10" s="57"/>
+      <c r="C10" s="57"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="57"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="57"/>
+      <c r="H10" s="56"/>
+      <c r="I10" s="56"/>
+      <c r="J10" s="56"/>
+      <c r="K10" s="56"/>
+      <c r="L10" s="56"/>
+      <c r="M10" s="56"/>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B11" s="57"/>
+      <c r="C11" s="57"/>
+      <c r="D11" s="57"/>
+      <c r="E11" s="57"/>
+      <c r="F11" s="57"/>
+      <c r="G11" s="57"/>
+      <c r="H11" s="56"/>
+      <c r="I11" s="56"/>
+      <c r="J11" s="56"/>
+      <c r="K11" s="56"/>
+      <c r="L11" s="56"/>
+      <c r="M11" s="56"/>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B12" s="55" t="s">
         <v>44</v>
       </c>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="42"/>
-      <c r="L2" s="42"/>
-      <c r="M2" s="42"/>
+      <c r="C12" s="55"/>
+      <c r="D12" s="55"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="56"/>
+      <c r="I12" s="56"/>
+      <c r="J12" s="56"/>
+      <c r="K12" s="56"/>
+      <c r="L12" s="56"/>
+      <c r="M12" s="56"/>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B3" s="43"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="42"/>
-      <c r="J3" s="42"/>
-      <c r="K3" s="42"/>
-      <c r="L3" s="42"/>
-      <c r="M3" s="42"/>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B13" s="57"/>
+      <c r="C13" s="57"/>
+      <c r="D13" s="57"/>
+      <c r="E13" s="57"/>
+      <c r="F13" s="57"/>
+      <c r="G13" s="57"/>
+      <c r="H13" s="56"/>
+      <c r="I13" s="56"/>
+      <c r="J13" s="56"/>
+      <c r="K13" s="56"/>
+      <c r="L13" s="56"/>
+      <c r="M13" s="56"/>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B4" s="43"/>
-      <c r="C4" s="43"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="43"/>
-      <c r="H4" s="42"/>
-      <c r="I4" s="42"/>
-      <c r="J4" s="42"/>
-      <c r="K4" s="42"/>
-      <c r="L4" s="42"/>
-      <c r="M4" s="42"/>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B14" s="57"/>
+      <c r="C14" s="57"/>
+      <c r="D14" s="57"/>
+      <c r="E14" s="57"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="57"/>
+      <c r="H14" s="56"/>
+      <c r="I14" s="56"/>
+      <c r="J14" s="56"/>
+      <c r="K14" s="56"/>
+      <c r="L14" s="56"/>
+      <c r="M14" s="56"/>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B5" s="41" t="s">
+    <row r="16" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B16" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="42"/>
-      <c r="K5" s="42"/>
-      <c r="L5" s="42"/>
-      <c r="M5" s="42"/>
+      <c r="C16" s="52"/>
+      <c r="D16" s="52"/>
+      <c r="E16" s="52"/>
+      <c r="F16" s="52"/>
+      <c r="G16" s="52"/>
+      <c r="H16" s="52"/>
+      <c r="I16" s="52"/>
+      <c r="J16" s="52"/>
+      <c r="K16" s="52"/>
+      <c r="L16" s="52"/>
+      <c r="M16" s="52"/>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B6" s="43"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="43"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="42"/>
-      <c r="I6" s="42"/>
-      <c r="J6" s="42"/>
-      <c r="K6" s="42"/>
-      <c r="L6" s="42"/>
-      <c r="M6" s="42"/>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B17" s="52"/>
+      <c r="C17" s="52"/>
+      <c r="D17" s="52"/>
+      <c r="E17" s="52"/>
+      <c r="F17" s="52"/>
+      <c r="G17" s="52"/>
+      <c r="H17" s="52"/>
+      <c r="I17" s="52"/>
+      <c r="J17" s="52"/>
+      <c r="K17" s="52"/>
+      <c r="L17" s="52"/>
+      <c r="M17" s="52"/>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="42"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="42"/>
-      <c r="K7" s="42"/>
-      <c r="L7" s="42"/>
-      <c r="M7" s="42"/>
-    </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B8" s="41" t="s">
-        <v>46</v>
-      </c>
-      <c r="C8" s="41"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="42"/>
-      <c r="I8" s="42"/>
-      <c r="J8" s="42"/>
-      <c r="K8" s="42"/>
-      <c r="L8" s="42"/>
-      <c r="M8" s="42"/>
-    </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B9" s="43"/>
-      <c r="C9" s="43"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="43"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="43"/>
-      <c r="H9" s="42"/>
-      <c r="I9" s="42"/>
-      <c r="J9" s="42"/>
-      <c r="K9" s="42"/>
-      <c r="L9" s="42"/>
-      <c r="M9" s="42"/>
-    </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B10" s="43"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="42"/>
-      <c r="I10" s="42"/>
-      <c r="J10" s="42"/>
-      <c r="K10" s="42"/>
-      <c r="L10" s="42"/>
-      <c r="M10" s="42"/>
-    </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
-      <c r="K11" s="42"/>
-      <c r="L11" s="42"/>
-      <c r="M11" s="42"/>
-    </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B12" s="41" t="s">
+    <row r="19" spans="2:13" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="B19" s="51" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
-      <c r="I12" s="42"/>
-      <c r="J12" s="42"/>
-      <c r="K12" s="42"/>
-      <c r="L12" s="42"/>
-      <c r="M12" s="42"/>
+      <c r="C19" s="51"/>
+      <c r="D19" s="51"/>
+      <c r="E19" s="51"/>
+      <c r="F19" s="51"/>
+      <c r="G19" s="51"/>
+      <c r="H19" s="51"/>
+      <c r="I19" s="51"/>
+      <c r="J19" s="51"/>
+      <c r="K19" s="51"/>
+      <c r="L19" s="51"/>
+      <c r="M19" s="51"/>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B13" s="43"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="42"/>
-      <c r="I13" s="42"/>
-      <c r="J13" s="42"/>
-      <c r="K13" s="42"/>
-      <c r="L13" s="42"/>
-      <c r="M13" s="42"/>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="24"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
+      <c r="L20" s="24"/>
+      <c r="M20" s="24"/>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B14" s="43"/>
-      <c r="C14" s="43"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="42"/>
-      <c r="I14" s="42"/>
-      <c r="J14" s="42"/>
-      <c r="K14" s="42"/>
-      <c r="L14" s="42"/>
-      <c r="M14" s="42"/>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="24"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="24"/>
+      <c r="L21" s="24"/>
+      <c r="M21" s="24"/>
     </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B16" s="38" t="s">
-        <v>48</v>
-      </c>
-      <c r="C16" s="38"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="38"/>
-      <c r="G16" s="38"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="38"/>
-      <c r="J16" s="38"/>
-      <c r="K16" s="38"/>
-      <c r="L16" s="38"/>
-      <c r="M16" s="38"/>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="24"/>
+      <c r="J22" s="24"/>
+      <c r="K22" s="24"/>
+      <c r="L22" s="24"/>
+      <c r="M22" s="24"/>
     </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="38"/>
-      <c r="G17" s="38"/>
-      <c r="H17" s="38"/>
-      <c r="I17" s="38"/>
-      <c r="J17" s="38"/>
-      <c r="K17" s="38"/>
-      <c r="L17" s="38"/>
-      <c r="M17" s="38"/>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="24"/>
+      <c r="J23" s="24"/>
+      <c r="K23" s="24"/>
+      <c r="L23" s="24"/>
+      <c r="M23" s="24"/>
     </row>
-    <row r="19" spans="2:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B19" s="59" t="s">
-        <v>50</v>
-      </c>
-      <c r="C19" s="59"/>
-      <c r="D19" s="59"/>
-      <c r="E19" s="59"/>
-      <c r="F19" s="59"/>
-      <c r="G19" s="59"/>
-      <c r="H19" s="59"/>
-      <c r="I19" s="59"/>
-      <c r="J19" s="59"/>
-      <c r="K19" s="59"/>
-      <c r="L19" s="59"/>
-      <c r="M19" s="59"/>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="24"/>
+      <c r="I24" s="24"/>
+      <c r="J24" s="24"/>
+      <c r="K24" s="24"/>
+      <c r="L24" s="24"/>
+      <c r="M24" s="24"/>
     </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B20" s="60"/>
-      <c r="C20" s="60"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
-      <c r="G20" s="60"/>
-      <c r="H20" s="60"/>
-      <c r="I20" s="60"/>
-      <c r="J20" s="60"/>
-      <c r="K20" s="60"/>
-      <c r="L20" s="60"/>
-      <c r="M20" s="60"/>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="24"/>
+      <c r="I25" s="24"/>
+      <c r="J25" s="24"/>
+      <c r="K25" s="24"/>
+      <c r="L25" s="24"/>
+      <c r="M25" s="24"/>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B21" s="60"/>
-      <c r="C21" s="60"/>
-      <c r="D21" s="60"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="60"/>
-      <c r="H21" s="60"/>
-      <c r="I21" s="60"/>
-      <c r="J21" s="60"/>
-      <c r="K21" s="60"/>
-      <c r="L21" s="60"/>
-      <c r="M21" s="60"/>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="24"/>
+      <c r="J26" s="24"/>
+      <c r="K26" s="24"/>
+      <c r="L26" s="24"/>
+      <c r="M26" s="24"/>
     </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B22" s="60"/>
-      <c r="C22" s="60"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="60"/>
-      <c r="G22" s="60"/>
-      <c r="H22" s="60"/>
-      <c r="I22" s="60"/>
-      <c r="J22" s="60"/>
-      <c r="K22" s="60"/>
-      <c r="L22" s="60"/>
-      <c r="M22" s="60"/>
+    <row r="27" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="24"/>
+      <c r="J27" s="24"/>
+      <c r="K27" s="24"/>
+      <c r="L27" s="24"/>
+      <c r="M27" s="24"/>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B23" s="60"/>
-      <c r="C23" s="60"/>
-      <c r="D23" s="60"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="60"/>
-      <c r="G23" s="60"/>
-      <c r="H23" s="60"/>
-      <c r="I23" s="60"/>
-      <c r="J23" s="60"/>
-      <c r="K23" s="60"/>
-      <c r="L23" s="60"/>
-      <c r="M23" s="60"/>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B28" s="24"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="24"/>
+      <c r="K28" s="24"/>
+      <c r="L28" s="24"/>
+      <c r="M28" s="24"/>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B24" s="60"/>
-      <c r="C24" s="60"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
-      <c r="G24" s="60"/>
-      <c r="H24" s="60"/>
-      <c r="I24" s="60"/>
-      <c r="J24" s="60"/>
-      <c r="K24" s="60"/>
-      <c r="L24" s="60"/>
-      <c r="M24" s="60"/>
+    <row r="29" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B29" s="24"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="24"/>
+      <c r="H29" s="24"/>
+      <c r="I29" s="24"/>
+      <c r="J29" s="24"/>
+      <c r="K29" s="24"/>
+      <c r="L29" s="24"/>
+      <c r="M29" s="24"/>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B25" s="60"/>
-      <c r="C25" s="60"/>
-      <c r="D25" s="60"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="60"/>
-      <c r="G25" s="60"/>
-      <c r="H25" s="60"/>
-      <c r="I25" s="60"/>
-      <c r="J25" s="60"/>
-      <c r="K25" s="60"/>
-      <c r="L25" s="60"/>
-      <c r="M25" s="60"/>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="24"/>
+      <c r="J30" s="24"/>
+      <c r="K30" s="24"/>
+      <c r="L30" s="24"/>
+      <c r="M30" s="24"/>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B26" s="60"/>
-      <c r="C26" s="60"/>
-      <c r="D26" s="60"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="60"/>
-      <c r="G26" s="60"/>
-      <c r="H26" s="60"/>
-      <c r="I26" s="60"/>
-      <c r="J26" s="60"/>
-      <c r="K26" s="60"/>
-      <c r="L26" s="60"/>
-      <c r="M26" s="60"/>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B31" s="24"/>
+      <c r="C31" s="24"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="24"/>
+      <c r="J31" s="24"/>
+      <c r="K31" s="24"/>
+      <c r="L31" s="24"/>
+      <c r="M31" s="24"/>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B27" s="60"/>
-      <c r="C27" s="60"/>
-      <c r="D27" s="60"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="60"/>
-      <c r="G27" s="60"/>
-      <c r="H27" s="60"/>
-      <c r="I27" s="60"/>
-      <c r="J27" s="60"/>
-      <c r="K27" s="60"/>
-      <c r="L27" s="60"/>
-      <c r="M27" s="60"/>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B32" s="24"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="24"/>
+      <c r="J32" s="24"/>
+      <c r="K32" s="24"/>
+      <c r="L32" s="24"/>
+      <c r="M32" s="24"/>
     </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B28" s="60"/>
-      <c r="C28" s="60"/>
-      <c r="D28" s="60"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="60"/>
-      <c r="G28" s="60"/>
-      <c r="H28" s="60"/>
-      <c r="I28" s="60"/>
-      <c r="J28" s="60"/>
-      <c r="K28" s="60"/>
-      <c r="L28" s="60"/>
-      <c r="M28" s="60"/>
+    <row r="33" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B33" s="24"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="24"/>
+      <c r="J33" s="24"/>
+      <c r="K33" s="24"/>
+      <c r="L33" s="24"/>
+      <c r="M33" s="24"/>
     </row>
-    <row r="29" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B29" s="60"/>
-      <c r="C29" s="60"/>
-      <c r="D29" s="60"/>
-      <c r="E29" s="60"/>
-      <c r="F29" s="60"/>
-      <c r="G29" s="60"/>
-      <c r="H29" s="60"/>
-      <c r="I29" s="60"/>
-      <c r="J29" s="60"/>
-      <c r="K29" s="60"/>
-      <c r="L29" s="60"/>
-      <c r="M29" s="60"/>
+    <row r="34" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B34" s="24"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="24"/>
+      <c r="J34" s="24"/>
+      <c r="K34" s="24"/>
+      <c r="L34" s="24"/>
+      <c r="M34" s="24"/>
     </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B30" s="60"/>
-      <c r="C30" s="60"/>
-      <c r="D30" s="60"/>
-      <c r="E30" s="60"/>
-      <c r="F30" s="60"/>
-      <c r="G30" s="60"/>
-      <c r="H30" s="60"/>
-      <c r="I30" s="60"/>
-      <c r="J30" s="60"/>
-      <c r="K30" s="60"/>
-      <c r="L30" s="60"/>
-      <c r="M30" s="60"/>
-    </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B31" s="60"/>
-      <c r="C31" s="60"/>
-      <c r="D31" s="60"/>
-      <c r="E31" s="60"/>
-      <c r="F31" s="60"/>
-      <c r="G31" s="60"/>
-      <c r="H31" s="60"/>
-      <c r="I31" s="60"/>
-      <c r="J31" s="60"/>
-      <c r="K31" s="60"/>
-      <c r="L31" s="60"/>
-      <c r="M31" s="60"/>
-    </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B32" s="60"/>
-      <c r="C32" s="60"/>
-      <c r="D32" s="60"/>
-      <c r="E32" s="60"/>
-      <c r="F32" s="60"/>
-      <c r="G32" s="60"/>
-      <c r="H32" s="60"/>
-      <c r="I32" s="60"/>
-      <c r="J32" s="60"/>
-      <c r="K32" s="60"/>
-      <c r="L32" s="60"/>
-      <c r="M32" s="60"/>
-    </row>
-    <row r="33" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B33" s="60"/>
-      <c r="C33" s="60"/>
-      <c r="D33" s="60"/>
-      <c r="E33" s="60"/>
-      <c r="F33" s="60"/>
-      <c r="G33" s="60"/>
-      <c r="H33" s="60"/>
-      <c r="I33" s="60"/>
-      <c r="J33" s="60"/>
-      <c r="K33" s="60"/>
-      <c r="L33" s="60"/>
-      <c r="M33" s="60"/>
-    </row>
-    <row r="34" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B34" s="60"/>
-      <c r="C34" s="60"/>
-      <c r="D34" s="60"/>
-      <c r="E34" s="60"/>
-      <c r="F34" s="60"/>
-      <c r="G34" s="60"/>
-      <c r="H34" s="60"/>
-      <c r="I34" s="60"/>
-      <c r="J34" s="60"/>
-      <c r="K34" s="60"/>
-      <c r="L34" s="60"/>
-      <c r="M34" s="60"/>
-    </row>
-    <row r="35" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B35" s="60"/>
-      <c r="C35" s="60"/>
-      <c r="D35" s="60"/>
-      <c r="E35" s="60"/>
-      <c r="F35" s="60"/>
-      <c r="G35" s="60"/>
-      <c r="H35" s="60"/>
-      <c r="I35" s="60"/>
-      <c r="J35" s="60"/>
-      <c r="K35" s="60"/>
-      <c r="L35" s="60"/>
-      <c r="M35" s="60"/>
+    <row r="35" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B35" s="24"/>
+      <c r="C35" s="24"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="24"/>
+      <c r="I35" s="24"/>
+      <c r="J35" s="24"/>
+      <c r="K35" s="24"/>
+      <c r="L35" s="24"/>
+      <c r="M35" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -22525,817 +22639,817 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D956047A-F1CE-4B2A-8F89-8CACF74DF670}">
   <dimension ref="A1:X31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A1" s="61" t="s">
-        <v>51</v>
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A1" s="21" t="s">
+        <v>48</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="61"/>
-      <c r="M1" s="61"/>
-      <c r="N1" s="61"/>
-      <c r="O1" s="61"/>
-      <c r="P1" s="61"/>
-      <c r="Q1" s="61"/>
-      <c r="R1" s="61"/>
-      <c r="S1" s="61"/>
-      <c r="T1" s="61"/>
-      <c r="U1" s="61"/>
-      <c r="V1" s="61"/>
-      <c r="W1" s="61"/>
-      <c r="X1" s="61"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
+      <c r="Q1" s="21"/>
+      <c r="R1" s="21"/>
+      <c r="S1" s="21"/>
+      <c r="T1" s="21"/>
+      <c r="U1" s="21"/>
+      <c r="V1" s="21"/>
+      <c r="W1" s="21"/>
+      <c r="X1" s="21"/>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A2" s="61"/>
-      <c r="B2" s="61"/>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
-      <c r="G2" s="61"/>
-      <c r="H2" s="61"/>
-      <c r="I2" s="61"/>
-      <c r="J2" s="61"/>
-      <c r="K2" s="61"/>
-      <c r="L2" s="61"/>
-      <c r="M2" s="61"/>
-      <c r="N2" s="61"/>
-      <c r="O2" s="61"/>
-      <c r="P2" s="61"/>
-      <c r="Q2" s="61"/>
-      <c r="R2" s="61"/>
-      <c r="S2" s="61"/>
-      <c r="T2" s="61"/>
-      <c r="U2" s="61"/>
-      <c r="V2" s="61"/>
-      <c r="W2" s="61"/>
-      <c r="X2" s="61"/>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A2" s="21"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
+      <c r="M2" s="21"/>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21"/>
+      <c r="P2" s="21"/>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="S2" s="21"/>
+      <c r="T2" s="21"/>
+      <c r="U2" s="21"/>
+      <c r="V2" s="21"/>
+      <c r="W2" s="21"/>
+      <c r="X2" s="21"/>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
-        <v>52</v>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A3" s="22" t="s">
+        <v>49</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
-      <c r="J3" s="63"/>
-      <c r="K3" s="63"/>
-      <c r="L3" s="63"/>
-      <c r="M3" s="63"/>
-      <c r="N3" s="63"/>
-      <c r="O3" s="63"/>
-      <c r="P3" s="63"/>
-      <c r="Q3" s="63"/>
-      <c r="R3" s="63"/>
-      <c r="S3" s="63"/>
-      <c r="T3" s="63"/>
-      <c r="U3" s="63"/>
-      <c r="V3" s="63"/>
-      <c r="W3" s="63"/>
-      <c r="X3" s="63"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="23"/>
+      <c r="R3" s="23"/>
+      <c r="S3" s="23"/>
+      <c r="T3" s="23"/>
+      <c r="U3" s="23"/>
+      <c r="V3" s="23"/>
+      <c r="W3" s="23"/>
+      <c r="X3" s="23"/>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A4" s="62"/>
-      <c r="B4" s="63"/>
-      <c r="C4" s="63"/>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="63"/>
-      <c r="L4" s="63"/>
-      <c r="M4" s="63"/>
-      <c r="N4" s="63"/>
-      <c r="O4" s="63"/>
-      <c r="P4" s="63"/>
-      <c r="Q4" s="63"/>
-      <c r="R4" s="63"/>
-      <c r="S4" s="63"/>
-      <c r="T4" s="63"/>
-      <c r="U4" s="63"/>
-      <c r="V4" s="63"/>
-      <c r="W4" s="63"/>
-      <c r="X4" s="63"/>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A4" s="22"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="23"/>
+      <c r="T4" s="23"/>
+      <c r="U4" s="23"/>
+      <c r="V4" s="23"/>
+      <c r="W4" s="23"/>
+      <c r="X4" s="23"/>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A5" s="62"/>
-      <c r="B5" s="63"/>
-      <c r="C5" s="63"/>
-      <c r="D5" s="63"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="63"/>
-      <c r="J5" s="63"/>
-      <c r="K5" s="63"/>
-      <c r="L5" s="63"/>
-      <c r="M5" s="63"/>
-      <c r="N5" s="63"/>
-      <c r="O5" s="63"/>
-      <c r="P5" s="63"/>
-      <c r="Q5" s="63"/>
-      <c r="R5" s="63"/>
-      <c r="S5" s="63"/>
-      <c r="T5" s="63"/>
-      <c r="U5" s="63"/>
-      <c r="V5" s="63"/>
-      <c r="W5" s="63"/>
-      <c r="X5" s="63"/>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A5" s="22"/>
+      <c r="B5" s="23"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="23"/>
+      <c r="L5" s="23"/>
+      <c r="M5" s="23"/>
+      <c r="N5" s="23"/>
+      <c r="O5" s="23"/>
+      <c r="P5" s="23"/>
+      <c r="Q5" s="23"/>
+      <c r="R5" s="23"/>
+      <c r="S5" s="23"/>
+      <c r="T5" s="23"/>
+      <c r="U5" s="23"/>
+      <c r="V5" s="23"/>
+      <c r="W5" s="23"/>
+      <c r="X5" s="23"/>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A6" s="60"/>
-      <c r="B6" s="60"/>
-      <c r="C6" s="60"/>
-      <c r="D6" s="60"/>
-      <c r="E6" s="60"/>
-      <c r="F6" s="60"/>
-      <c r="G6" s="60"/>
-      <c r="H6" s="60"/>
-      <c r="I6" s="60"/>
-      <c r="J6" s="60"/>
-      <c r="K6" s="60"/>
-      <c r="L6" s="60"/>
-      <c r="M6" s="60"/>
-      <c r="N6" s="60"/>
-      <c r="O6" s="60"/>
-      <c r="P6" s="60"/>
-      <c r="Q6" s="60"/>
-      <c r="R6" s="60"/>
-      <c r="S6" s="60"/>
-      <c r="T6" s="60"/>
-      <c r="U6" s="60"/>
-      <c r="V6" s="60"/>
-      <c r="W6" s="60"/>
-      <c r="X6" s="60"/>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A6" s="24"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="24"/>
+      <c r="M6" s="24"/>
+      <c r="N6" s="24"/>
+      <c r="O6" s="24"/>
+      <c r="P6" s="24"/>
+      <c r="Q6" s="24"/>
+      <c r="R6" s="24"/>
+      <c r="S6" s="24"/>
+      <c r="T6" s="24"/>
+      <c r="U6" s="24"/>
+      <c r="V6" s="24"/>
+      <c r="W6" s="24"/>
+      <c r="X6" s="24"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A7" s="60"/>
-      <c r="B7" s="60"/>
-      <c r="C7" s="60"/>
-      <c r="D7" s="60"/>
-      <c r="E7" s="60"/>
-      <c r="F7" s="60"/>
-      <c r="G7" s="60"/>
-      <c r="H7" s="60"/>
-      <c r="I7" s="60"/>
-      <c r="J7" s="60"/>
-      <c r="K7" s="60"/>
-      <c r="L7" s="60"/>
-      <c r="M7" s="60"/>
-      <c r="N7" s="60"/>
-      <c r="O7" s="60"/>
-      <c r="P7" s="60"/>
-      <c r="Q7" s="60"/>
-      <c r="R7" s="60"/>
-      <c r="S7" s="60"/>
-      <c r="T7" s="60"/>
-      <c r="U7" s="60"/>
-      <c r="V7" s="60"/>
-      <c r="W7" s="60"/>
-      <c r="X7" s="60"/>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A7" s="24"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="24"/>
+      <c r="K7" s="24"/>
+      <c r="L7" s="24"/>
+      <c r="M7" s="24"/>
+      <c r="N7" s="24"/>
+      <c r="O7" s="24"/>
+      <c r="P7" s="24"/>
+      <c r="Q7" s="24"/>
+      <c r="R7" s="24"/>
+      <c r="S7" s="24"/>
+      <c r="T7" s="24"/>
+      <c r="U7" s="24"/>
+      <c r="V7" s="24"/>
+      <c r="W7" s="24"/>
+      <c r="X7" s="24"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A8" s="60"/>
-      <c r="B8" s="60"/>
-      <c r="C8" s="60"/>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="60"/>
-      <c r="G8" s="60"/>
-      <c r="H8" s="60"/>
-      <c r="I8" s="60"/>
-      <c r="J8" s="60"/>
-      <c r="K8" s="60"/>
-      <c r="L8" s="60"/>
-      <c r="M8" s="60"/>
-      <c r="N8" s="60"/>
-      <c r="O8" s="60"/>
-      <c r="P8" s="60"/>
-      <c r="Q8" s="60"/>
-      <c r="R8" s="60"/>
-      <c r="S8" s="60"/>
-      <c r="T8" s="60"/>
-      <c r="U8" s="60"/>
-      <c r="V8" s="60"/>
-      <c r="W8" s="60"/>
-      <c r="X8" s="60"/>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A8" s="24"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
+      <c r="I8" s="24"/>
+      <c r="J8" s="24"/>
+      <c r="K8" s="24"/>
+      <c r="L8" s="24"/>
+      <c r="M8" s="24"/>
+      <c r="N8" s="24"/>
+      <c r="O8" s="24"/>
+      <c r="P8" s="24"/>
+      <c r="Q8" s="24"/>
+      <c r="R8" s="24"/>
+      <c r="S8" s="24"/>
+      <c r="T8" s="24"/>
+      <c r="U8" s="24"/>
+      <c r="V8" s="24"/>
+      <c r="W8" s="24"/>
+      <c r="X8" s="24"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A9" s="60"/>
-      <c r="B9" s="60"/>
-      <c r="C9" s="60"/>
-      <c r="D9" s="60"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="60"/>
-      <c r="G9" s="60"/>
-      <c r="H9" s="60"/>
-      <c r="I9" s="60"/>
-      <c r="J9" s="60"/>
-      <c r="K9" s="60"/>
-      <c r="L9" s="60"/>
-      <c r="M9" s="60"/>
-      <c r="N9" s="60"/>
-      <c r="O9" s="60"/>
-      <c r="P9" s="60"/>
-      <c r="Q9" s="60"/>
-      <c r="R9" s="60"/>
-      <c r="S9" s="60"/>
-      <c r="T9" s="60"/>
-      <c r="U9" s="60"/>
-      <c r="V9" s="60"/>
-      <c r="W9" s="60"/>
-      <c r="X9" s="60"/>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A9" s="24"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="24"/>
+      <c r="J9" s="24"/>
+      <c r="K9" s="24"/>
+      <c r="L9" s="24"/>
+      <c r="M9" s="24"/>
+      <c r="N9" s="24"/>
+      <c r="O9" s="24"/>
+      <c r="P9" s="24"/>
+      <c r="Q9" s="24"/>
+      <c r="R9" s="24"/>
+      <c r="S9" s="24"/>
+      <c r="T9" s="24"/>
+      <c r="U9" s="24"/>
+      <c r="V9" s="24"/>
+      <c r="W9" s="24"/>
+      <c r="X9" s="24"/>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A10" s="60"/>
-      <c r="B10" s="60"/>
-      <c r="C10" s="60"/>
-      <c r="D10" s="60"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="60"/>
-      <c r="G10" s="60"/>
-      <c r="H10" s="60"/>
-      <c r="I10" s="60"/>
-      <c r="J10" s="60"/>
-      <c r="K10" s="60"/>
-      <c r="L10" s="60"/>
-      <c r="M10" s="60"/>
-      <c r="N10" s="60"/>
-      <c r="O10" s="60"/>
-      <c r="P10" s="60"/>
-      <c r="Q10" s="60"/>
-      <c r="R10" s="60"/>
-      <c r="S10" s="60"/>
-      <c r="T10" s="60"/>
-      <c r="U10" s="60"/>
-      <c r="V10" s="60"/>
-      <c r="W10" s="60"/>
-      <c r="X10" s="60"/>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="24"/>
+      <c r="L10" s="24"/>
+      <c r="M10" s="24"/>
+      <c r="N10" s="24"/>
+      <c r="O10" s="24"/>
+      <c r="P10" s="24"/>
+      <c r="Q10" s="24"/>
+      <c r="R10" s="24"/>
+      <c r="S10" s="24"/>
+      <c r="T10" s="24"/>
+      <c r="U10" s="24"/>
+      <c r="V10" s="24"/>
+      <c r="W10" s="24"/>
+      <c r="X10" s="24"/>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A11" s="60"/>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
-      <c r="J11" s="60"/>
-      <c r="K11" s="60"/>
-      <c r="L11" s="60"/>
-      <c r="M11" s="60"/>
-      <c r="N11" s="60"/>
-      <c r="O11" s="60"/>
-      <c r="P11" s="60"/>
-      <c r="Q11" s="60"/>
-      <c r="R11" s="60"/>
-      <c r="S11" s="60"/>
-      <c r="T11" s="60"/>
-      <c r="U11" s="60"/>
-      <c r="V11" s="60"/>
-      <c r="W11" s="60"/>
-      <c r="X11" s="60"/>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A11" s="24"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="24"/>
+      <c r="K11" s="24"/>
+      <c r="L11" s="24"/>
+      <c r="M11" s="24"/>
+      <c r="N11" s="24"/>
+      <c r="O11" s="24"/>
+      <c r="P11" s="24"/>
+      <c r="Q11" s="24"/>
+      <c r="R11" s="24"/>
+      <c r="S11" s="24"/>
+      <c r="T11" s="24"/>
+      <c r="U11" s="24"/>
+      <c r="V11" s="24"/>
+      <c r="W11" s="24"/>
+      <c r="X11" s="24"/>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A12" s="60"/>
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="60"/>
-      <c r="J12" s="60"/>
-      <c r="K12" s="60"/>
-      <c r="L12" s="60"/>
-      <c r="M12" s="60"/>
-      <c r="N12" s="60"/>
-      <c r="O12" s="60"/>
-      <c r="P12" s="60"/>
-      <c r="Q12" s="60"/>
-      <c r="R12" s="60"/>
-      <c r="S12" s="60"/>
-      <c r="T12" s="60"/>
-      <c r="U12" s="60"/>
-      <c r="V12" s="60"/>
-      <c r="W12" s="60"/>
-      <c r="X12" s="60"/>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A12" s="24"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="24"/>
+      <c r="L12" s="24"/>
+      <c r="M12" s="24"/>
+      <c r="N12" s="24"/>
+      <c r="O12" s="24"/>
+      <c r="P12" s="24"/>
+      <c r="Q12" s="24"/>
+      <c r="R12" s="24"/>
+      <c r="S12" s="24"/>
+      <c r="T12" s="24"/>
+      <c r="U12" s="24"/>
+      <c r="V12" s="24"/>
+      <c r="W12" s="24"/>
+      <c r="X12" s="24"/>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A13" s="60"/>
-      <c r="B13" s="60"/>
-      <c r="C13" s="60"/>
-      <c r="D13" s="60"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="60"/>
-      <c r="H13" s="60"/>
-      <c r="I13" s="60"/>
-      <c r="J13" s="60"/>
-      <c r="K13" s="60"/>
-      <c r="L13" s="60"/>
-      <c r="M13" s="60"/>
-      <c r="N13" s="60"/>
-      <c r="O13" s="60"/>
-      <c r="P13" s="60"/>
-      <c r="Q13" s="60"/>
-      <c r="R13" s="60"/>
-      <c r="S13" s="60"/>
-      <c r="T13" s="60"/>
-      <c r="U13" s="60"/>
-      <c r="V13" s="60"/>
-      <c r="W13" s="60"/>
-      <c r="X13" s="60"/>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A13" s="24"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="24"/>
+      <c r="J13" s="24"/>
+      <c r="K13" s="24"/>
+      <c r="L13" s="24"/>
+      <c r="M13" s="24"/>
+      <c r="N13" s="24"/>
+      <c r="O13" s="24"/>
+      <c r="P13" s="24"/>
+      <c r="Q13" s="24"/>
+      <c r="R13" s="24"/>
+      <c r="S13" s="24"/>
+      <c r="T13" s="24"/>
+      <c r="U13" s="24"/>
+      <c r="V13" s="24"/>
+      <c r="W13" s="24"/>
+      <c r="X13" s="24"/>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A14" s="60"/>
-      <c r="B14" s="60"/>
-      <c r="C14" s="60"/>
-      <c r="D14" s="60"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="60"/>
-      <c r="G14" s="60"/>
-      <c r="H14" s="60"/>
-      <c r="I14" s="60"/>
-      <c r="J14" s="60"/>
-      <c r="K14" s="60"/>
-      <c r="L14" s="60"/>
-      <c r="M14" s="60"/>
-      <c r="N14" s="60"/>
-      <c r="O14" s="60"/>
-      <c r="P14" s="60"/>
-      <c r="Q14" s="60"/>
-      <c r="R14" s="60"/>
-      <c r="S14" s="60"/>
-      <c r="T14" s="60"/>
-      <c r="U14" s="60"/>
-      <c r="V14" s="60"/>
-      <c r="W14" s="60"/>
-      <c r="X14" s="60"/>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A14" s="24"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="24"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="24"/>
+      <c r="L14" s="24"/>
+      <c r="M14" s="24"/>
+      <c r="N14" s="24"/>
+      <c r="O14" s="24"/>
+      <c r="P14" s="24"/>
+      <c r="Q14" s="24"/>
+      <c r="R14" s="24"/>
+      <c r="S14" s="24"/>
+      <c r="T14" s="24"/>
+      <c r="U14" s="24"/>
+      <c r="V14" s="24"/>
+      <c r="W14" s="24"/>
+      <c r="X14" s="24"/>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A15" s="60"/>
-      <c r="B15" s="60"/>
-      <c r="C15" s="60"/>
-      <c r="D15" s="60"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
-      <c r="G15" s="60"/>
-      <c r="H15" s="60"/>
-      <c r="I15" s="60"/>
-      <c r="J15" s="60"/>
-      <c r="K15" s="60"/>
-      <c r="L15" s="60"/>
-      <c r="M15" s="60"/>
-      <c r="N15" s="60"/>
-      <c r="O15" s="60"/>
-      <c r="P15" s="60"/>
-      <c r="Q15" s="60"/>
-      <c r="R15" s="60"/>
-      <c r="S15" s="60"/>
-      <c r="T15" s="60"/>
-      <c r="U15" s="60"/>
-      <c r="V15" s="60"/>
-      <c r="W15" s="60"/>
-      <c r="X15" s="60"/>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A15" s="24"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="24"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="24"/>
+      <c r="L15" s="24"/>
+      <c r="M15" s="24"/>
+      <c r="N15" s="24"/>
+      <c r="O15" s="24"/>
+      <c r="P15" s="24"/>
+      <c r="Q15" s="24"/>
+      <c r="R15" s="24"/>
+      <c r="S15" s="24"/>
+      <c r="T15" s="24"/>
+      <c r="U15" s="24"/>
+      <c r="V15" s="24"/>
+      <c r="W15" s="24"/>
+      <c r="X15" s="24"/>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A16" s="60"/>
-      <c r="B16" s="60"/>
-      <c r="C16" s="60"/>
-      <c r="D16" s="60"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="60"/>
-      <c r="G16" s="60"/>
-      <c r="H16" s="60"/>
-      <c r="I16" s="60"/>
-      <c r="J16" s="60"/>
-      <c r="K16" s="60"/>
-      <c r="L16" s="60"/>
-      <c r="M16" s="60"/>
-      <c r="N16" s="60"/>
-      <c r="O16" s="60"/>
-      <c r="P16" s="60"/>
-      <c r="Q16" s="60"/>
-      <c r="R16" s="60"/>
-      <c r="S16" s="60"/>
-      <c r="T16" s="60"/>
-      <c r="U16" s="60"/>
-      <c r="V16" s="60"/>
-      <c r="W16" s="60"/>
-      <c r="X16" s="60"/>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A16" s="24"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
+      <c r="L16" s="24"/>
+      <c r="M16" s="24"/>
+      <c r="N16" s="24"/>
+      <c r="O16" s="24"/>
+      <c r="P16" s="24"/>
+      <c r="Q16" s="24"/>
+      <c r="R16" s="24"/>
+      <c r="S16" s="24"/>
+      <c r="T16" s="24"/>
+      <c r="U16" s="24"/>
+      <c r="V16" s="24"/>
+      <c r="W16" s="24"/>
+      <c r="X16" s="24"/>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A17" s="60"/>
-      <c r="B17" s="60"/>
-      <c r="C17" s="60"/>
-      <c r="D17" s="60"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="60"/>
-      <c r="H17" s="60"/>
-      <c r="I17" s="60"/>
-      <c r="J17" s="60"/>
-      <c r="K17" s="60"/>
-      <c r="L17" s="60"/>
-      <c r="M17" s="60"/>
-      <c r="N17" s="60"/>
-      <c r="O17" s="60"/>
-      <c r="P17" s="60"/>
-      <c r="Q17" s="60"/>
-      <c r="R17" s="60"/>
-      <c r="S17" s="60"/>
-      <c r="T17" s="60"/>
-      <c r="U17" s="60"/>
-      <c r="V17" s="60"/>
-      <c r="W17" s="60"/>
-      <c r="X17" s="60"/>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A17" s="24"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="24"/>
+      <c r="J17" s="24"/>
+      <c r="K17" s="24"/>
+      <c r="L17" s="24"/>
+      <c r="M17" s="24"/>
+      <c r="N17" s="24"/>
+      <c r="O17" s="24"/>
+      <c r="P17" s="24"/>
+      <c r="Q17" s="24"/>
+      <c r="R17" s="24"/>
+      <c r="S17" s="24"/>
+      <c r="T17" s="24"/>
+      <c r="U17" s="24"/>
+      <c r="V17" s="24"/>
+      <c r="W17" s="24"/>
+      <c r="X17" s="24"/>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A18" s="60"/>
-      <c r="B18" s="60"/>
-      <c r="C18" s="60"/>
-      <c r="D18" s="60"/>
-      <c r="E18" s="60"/>
-      <c r="F18" s="60"/>
-      <c r="G18" s="60"/>
-      <c r="H18" s="60"/>
-      <c r="I18" s="60"/>
-      <c r="J18" s="60"/>
-      <c r="K18" s="60"/>
-      <c r="L18" s="60"/>
-      <c r="M18" s="60"/>
-      <c r="N18" s="60"/>
-      <c r="O18" s="60"/>
-      <c r="P18" s="60"/>
-      <c r="Q18" s="60"/>
-      <c r="R18" s="60"/>
-      <c r="S18" s="60"/>
-      <c r="T18" s="60"/>
-      <c r="U18" s="60"/>
-      <c r="V18" s="60"/>
-      <c r="W18" s="60"/>
-      <c r="X18" s="60"/>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A18" s="24"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="24"/>
+      <c r="L18" s="24"/>
+      <c r="M18" s="24"/>
+      <c r="N18" s="24"/>
+      <c r="O18" s="24"/>
+      <c r="P18" s="24"/>
+      <c r="Q18" s="24"/>
+      <c r="R18" s="24"/>
+      <c r="S18" s="24"/>
+      <c r="T18" s="24"/>
+      <c r="U18" s="24"/>
+      <c r="V18" s="24"/>
+      <c r="W18" s="24"/>
+      <c r="X18" s="24"/>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A19" s="60"/>
-      <c r="B19" s="60"/>
-      <c r="C19" s="60"/>
-      <c r="D19" s="60"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="60"/>
-      <c r="G19" s="60"/>
-      <c r="H19" s="60"/>
-      <c r="I19" s="60"/>
-      <c r="J19" s="60"/>
-      <c r="K19" s="60"/>
-      <c r="L19" s="60"/>
-      <c r="M19" s="60"/>
-      <c r="N19" s="60"/>
-      <c r="O19" s="60"/>
-      <c r="P19" s="60"/>
-      <c r="Q19" s="60"/>
-      <c r="R19" s="60"/>
-      <c r="S19" s="60"/>
-      <c r="T19" s="60"/>
-      <c r="U19" s="60"/>
-      <c r="V19" s="60"/>
-      <c r="W19" s="60"/>
-      <c r="X19" s="60"/>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A19" s="24"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="24"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="24"/>
+      <c r="K19" s="24"/>
+      <c r="L19" s="24"/>
+      <c r="M19" s="24"/>
+      <c r="N19" s="24"/>
+      <c r="O19" s="24"/>
+      <c r="P19" s="24"/>
+      <c r="Q19" s="24"/>
+      <c r="R19" s="24"/>
+      <c r="S19" s="24"/>
+      <c r="T19" s="24"/>
+      <c r="U19" s="24"/>
+      <c r="V19" s="24"/>
+      <c r="W19" s="24"/>
+      <c r="X19" s="24"/>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A20" s="60"/>
-      <c r="B20" s="60"/>
-      <c r="C20" s="60"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
-      <c r="G20" s="60"/>
-      <c r="H20" s="60"/>
-      <c r="I20" s="60"/>
-      <c r="J20" s="60"/>
-      <c r="K20" s="60"/>
-      <c r="L20" s="60"/>
-      <c r="M20" s="60"/>
-      <c r="N20" s="60"/>
-      <c r="O20" s="60"/>
-      <c r="P20" s="60"/>
-      <c r="Q20" s="60"/>
-      <c r="R20" s="60"/>
-      <c r="S20" s="60"/>
-      <c r="T20" s="60"/>
-      <c r="U20" s="60"/>
-      <c r="V20" s="60"/>
-      <c r="W20" s="60"/>
-      <c r="X20" s="60"/>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A20" s="24"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="24"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
+      <c r="L20" s="24"/>
+      <c r="M20" s="24"/>
+      <c r="N20" s="24"/>
+      <c r="O20" s="24"/>
+      <c r="P20" s="24"/>
+      <c r="Q20" s="24"/>
+      <c r="R20" s="24"/>
+      <c r="S20" s="24"/>
+      <c r="T20" s="24"/>
+      <c r="U20" s="24"/>
+      <c r="V20" s="24"/>
+      <c r="W20" s="24"/>
+      <c r="X20" s="24"/>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A21" s="60"/>
-      <c r="B21" s="60"/>
-      <c r="C21" s="60"/>
-      <c r="D21" s="60"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="60"/>
-      <c r="H21" s="60"/>
-      <c r="I21" s="60"/>
-      <c r="J21" s="60"/>
-      <c r="K21" s="60"/>
-      <c r="L21" s="60"/>
-      <c r="M21" s="60"/>
-      <c r="N21" s="60"/>
-      <c r="O21" s="60"/>
-      <c r="P21" s="60"/>
-      <c r="Q21" s="60"/>
-      <c r="R21" s="60"/>
-      <c r="S21" s="60"/>
-      <c r="T21" s="60"/>
-      <c r="U21" s="60"/>
-      <c r="V21" s="60"/>
-      <c r="W21" s="60"/>
-      <c r="X21" s="60"/>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A21" s="24"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="24"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="24"/>
+      <c r="L21" s="24"/>
+      <c r="M21" s="24"/>
+      <c r="N21" s="24"/>
+      <c r="O21" s="24"/>
+      <c r="P21" s="24"/>
+      <c r="Q21" s="24"/>
+      <c r="R21" s="24"/>
+      <c r="S21" s="24"/>
+      <c r="T21" s="24"/>
+      <c r="U21" s="24"/>
+      <c r="V21" s="24"/>
+      <c r="W21" s="24"/>
+      <c r="X21" s="24"/>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A22" s="60"/>
-      <c r="B22" s="60"/>
-      <c r="C22" s="60"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="60"/>
-      <c r="G22" s="60"/>
-      <c r="H22" s="60"/>
-      <c r="I22" s="60"/>
-      <c r="J22" s="60"/>
-      <c r="K22" s="60"/>
-      <c r="L22" s="60"/>
-      <c r="M22" s="60"/>
-      <c r="N22" s="60"/>
-      <c r="O22" s="60"/>
-      <c r="P22" s="60"/>
-      <c r="Q22" s="60"/>
-      <c r="R22" s="60"/>
-      <c r="S22" s="60"/>
-      <c r="T22" s="60"/>
-      <c r="U22" s="60"/>
-      <c r="V22" s="60"/>
-      <c r="W22" s="60"/>
-      <c r="X22" s="60"/>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A22" s="24"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="24"/>
+      <c r="J22" s="24"/>
+      <c r="K22" s="24"/>
+      <c r="L22" s="24"/>
+      <c r="M22" s="24"/>
+      <c r="N22" s="24"/>
+      <c r="O22" s="24"/>
+      <c r="P22" s="24"/>
+      <c r="Q22" s="24"/>
+      <c r="R22" s="24"/>
+      <c r="S22" s="24"/>
+      <c r="T22" s="24"/>
+      <c r="U22" s="24"/>
+      <c r="V22" s="24"/>
+      <c r="W22" s="24"/>
+      <c r="X22" s="24"/>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A23" s="60"/>
-      <c r="B23" s="60"/>
-      <c r="C23" s="60"/>
-      <c r="D23" s="60"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="60"/>
-      <c r="G23" s="60"/>
-      <c r="H23" s="60"/>
-      <c r="I23" s="60"/>
-      <c r="J23" s="60"/>
-      <c r="K23" s="60"/>
-      <c r="L23" s="60"/>
-      <c r="M23" s="60"/>
-      <c r="N23" s="60"/>
-      <c r="O23" s="60"/>
-      <c r="P23" s="60"/>
-      <c r="Q23" s="60"/>
-      <c r="R23" s="60"/>
-      <c r="S23" s="60"/>
-      <c r="T23" s="60"/>
-      <c r="U23" s="60"/>
-      <c r="V23" s="60"/>
-      <c r="W23" s="60"/>
-      <c r="X23" s="60"/>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A23" s="24"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="24"/>
+      <c r="J23" s="24"/>
+      <c r="K23" s="24"/>
+      <c r="L23" s="24"/>
+      <c r="M23" s="24"/>
+      <c r="N23" s="24"/>
+      <c r="O23" s="24"/>
+      <c r="P23" s="24"/>
+      <c r="Q23" s="24"/>
+      <c r="R23" s="24"/>
+      <c r="S23" s="24"/>
+      <c r="T23" s="24"/>
+      <c r="U23" s="24"/>
+      <c r="V23" s="24"/>
+      <c r="W23" s="24"/>
+      <c r="X23" s="24"/>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A24" s="60"/>
-      <c r="B24" s="60"/>
-      <c r="C24" s="60"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
-      <c r="G24" s="60"/>
-      <c r="H24" s="60"/>
-      <c r="I24" s="60"/>
-      <c r="J24" s="60"/>
-      <c r="K24" s="60"/>
-      <c r="L24" s="60"/>
-      <c r="M24" s="60"/>
-      <c r="N24" s="60"/>
-      <c r="O24" s="60"/>
-      <c r="P24" s="60"/>
-      <c r="Q24" s="60"/>
-      <c r="R24" s="60"/>
-      <c r="S24" s="60"/>
-      <c r="T24" s="60"/>
-      <c r="U24" s="60"/>
-      <c r="V24" s="60"/>
-      <c r="W24" s="60"/>
-      <c r="X24" s="60"/>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A24" s="24"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="24"/>
+      <c r="I24" s="24"/>
+      <c r="J24" s="24"/>
+      <c r="K24" s="24"/>
+      <c r="L24" s="24"/>
+      <c r="M24" s="24"/>
+      <c r="N24" s="24"/>
+      <c r="O24" s="24"/>
+      <c r="P24" s="24"/>
+      <c r="Q24" s="24"/>
+      <c r="R24" s="24"/>
+      <c r="S24" s="24"/>
+      <c r="T24" s="24"/>
+      <c r="U24" s="24"/>
+      <c r="V24" s="24"/>
+      <c r="W24" s="24"/>
+      <c r="X24" s="24"/>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A25" s="60"/>
-      <c r="B25" s="60"/>
-      <c r="C25" s="60"/>
-      <c r="D25" s="60"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="60"/>
-      <c r="G25" s="60"/>
-      <c r="H25" s="60"/>
-      <c r="I25" s="60"/>
-      <c r="J25" s="60"/>
-      <c r="K25" s="60"/>
-      <c r="L25" s="60"/>
-      <c r="M25" s="60"/>
-      <c r="N25" s="60"/>
-      <c r="O25" s="60"/>
-      <c r="P25" s="60"/>
-      <c r="Q25" s="60"/>
-      <c r="R25" s="60"/>
-      <c r="S25" s="60"/>
-      <c r="T25" s="60"/>
-      <c r="U25" s="60"/>
-      <c r="V25" s="60"/>
-      <c r="W25" s="60"/>
-      <c r="X25" s="60"/>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A25" s="24"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="24"/>
+      <c r="I25" s="24"/>
+      <c r="J25" s="24"/>
+      <c r="K25" s="24"/>
+      <c r="L25" s="24"/>
+      <c r="M25" s="24"/>
+      <c r="N25" s="24"/>
+      <c r="O25" s="24"/>
+      <c r="P25" s="24"/>
+      <c r="Q25" s="24"/>
+      <c r="R25" s="24"/>
+      <c r="S25" s="24"/>
+      <c r="T25" s="24"/>
+      <c r="U25" s="24"/>
+      <c r="V25" s="24"/>
+      <c r="W25" s="24"/>
+      <c r="X25" s="24"/>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A26" s="60"/>
-      <c r="B26" s="60"/>
-      <c r="C26" s="60"/>
-      <c r="D26" s="60"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="60"/>
-      <c r="G26" s="60"/>
-      <c r="H26" s="60"/>
-      <c r="I26" s="60"/>
-      <c r="J26" s="60"/>
-      <c r="K26" s="60"/>
-      <c r="L26" s="60"/>
-      <c r="M26" s="60"/>
-      <c r="N26" s="60"/>
-      <c r="O26" s="60"/>
-      <c r="P26" s="60"/>
-      <c r="Q26" s="60"/>
-      <c r="R26" s="60"/>
-      <c r="S26" s="60"/>
-      <c r="T26" s="60"/>
-      <c r="U26" s="60"/>
-      <c r="V26" s="60"/>
-      <c r="W26" s="60"/>
-      <c r="X26" s="60"/>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A26" s="24"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="24"/>
+      <c r="J26" s="24"/>
+      <c r="K26" s="24"/>
+      <c r="L26" s="24"/>
+      <c r="M26" s="24"/>
+      <c r="N26" s="24"/>
+      <c r="O26" s="24"/>
+      <c r="P26" s="24"/>
+      <c r="Q26" s="24"/>
+      <c r="R26" s="24"/>
+      <c r="S26" s="24"/>
+      <c r="T26" s="24"/>
+      <c r="U26" s="24"/>
+      <c r="V26" s="24"/>
+      <c r="W26" s="24"/>
+      <c r="X26" s="24"/>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A27" s="60"/>
-      <c r="B27" s="60"/>
-      <c r="C27" s="60"/>
-      <c r="D27" s="60"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="60"/>
-      <c r="G27" s="60"/>
-      <c r="H27" s="60"/>
-      <c r="I27" s="60"/>
-      <c r="J27" s="60"/>
-      <c r="K27" s="60"/>
-      <c r="L27" s="60"/>
-      <c r="M27" s="60"/>
-      <c r="N27" s="60"/>
-      <c r="O27" s="60"/>
-      <c r="P27" s="60"/>
-      <c r="Q27" s="60"/>
-      <c r="R27" s="60"/>
-      <c r="S27" s="60"/>
-      <c r="T27" s="60"/>
-      <c r="U27" s="60"/>
-      <c r="V27" s="60"/>
-      <c r="W27" s="60"/>
-      <c r="X27" s="60"/>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A27" s="24"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="24"/>
+      <c r="J27" s="24"/>
+      <c r="K27" s="24"/>
+      <c r="L27" s="24"/>
+      <c r="M27" s="24"/>
+      <c r="N27" s="24"/>
+      <c r="O27" s="24"/>
+      <c r="P27" s="24"/>
+      <c r="Q27" s="24"/>
+      <c r="R27" s="24"/>
+      <c r="S27" s="24"/>
+      <c r="T27" s="24"/>
+      <c r="U27" s="24"/>
+      <c r="V27" s="24"/>
+      <c r="W27" s="24"/>
+      <c r="X27" s="24"/>
     </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A28" s="60"/>
-      <c r="B28" s="60"/>
-      <c r="C28" s="60"/>
-      <c r="D28" s="60"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="60"/>
-      <c r="G28" s="60"/>
-      <c r="H28" s="60"/>
-      <c r="I28" s="60"/>
-      <c r="J28" s="60"/>
-      <c r="K28" s="60"/>
-      <c r="L28" s="60"/>
-      <c r="M28" s="60"/>
-      <c r="N28" s="60"/>
-      <c r="O28" s="60"/>
-      <c r="P28" s="60"/>
-      <c r="Q28" s="60"/>
-      <c r="R28" s="60"/>
-      <c r="S28" s="60"/>
-      <c r="T28" s="60"/>
-      <c r="U28" s="60"/>
-      <c r="V28" s="60"/>
-      <c r="W28" s="60"/>
-      <c r="X28" s="60"/>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A28" s="24"/>
+      <c r="B28" s="24"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="24"/>
+      <c r="K28" s="24"/>
+      <c r="L28" s="24"/>
+      <c r="M28" s="24"/>
+      <c r="N28" s="24"/>
+      <c r="O28" s="24"/>
+      <c r="P28" s="24"/>
+      <c r="Q28" s="24"/>
+      <c r="R28" s="24"/>
+      <c r="S28" s="24"/>
+      <c r="T28" s="24"/>
+      <c r="U28" s="24"/>
+      <c r="V28" s="24"/>
+      <c r="W28" s="24"/>
+      <c r="X28" s="24"/>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A29" s="60"/>
-      <c r="B29" s="60"/>
-      <c r="C29" s="60"/>
-      <c r="D29" s="60"/>
-      <c r="E29" s="60"/>
-      <c r="F29" s="60"/>
-      <c r="G29" s="60"/>
-      <c r="H29" s="60"/>
-      <c r="I29" s="60"/>
-      <c r="J29" s="60"/>
-      <c r="K29" s="60"/>
-      <c r="L29" s="60"/>
-      <c r="M29" s="60"/>
-      <c r="N29" s="60"/>
-      <c r="O29" s="60"/>
-      <c r="P29" s="60"/>
-      <c r="Q29" s="60"/>
-      <c r="R29" s="60"/>
-      <c r="S29" s="60"/>
-      <c r="T29" s="60"/>
-      <c r="U29" s="60"/>
-      <c r="V29" s="60"/>
-      <c r="W29" s="60"/>
-      <c r="X29" s="60"/>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A29" s="24"/>
+      <c r="B29" s="24"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="24"/>
+      <c r="H29" s="24"/>
+      <c r="I29" s="24"/>
+      <c r="J29" s="24"/>
+      <c r="K29" s="24"/>
+      <c r="L29" s="24"/>
+      <c r="M29" s="24"/>
+      <c r="N29" s="24"/>
+      <c r="O29" s="24"/>
+      <c r="P29" s="24"/>
+      <c r="Q29" s="24"/>
+      <c r="R29" s="24"/>
+      <c r="S29" s="24"/>
+      <c r="T29" s="24"/>
+      <c r="U29" s="24"/>
+      <c r="V29" s="24"/>
+      <c r="W29" s="24"/>
+      <c r="X29" s="24"/>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A30" s="60"/>
-      <c r="B30" s="60"/>
-      <c r="C30" s="60"/>
-      <c r="D30" s="60"/>
-      <c r="E30" s="60"/>
-      <c r="F30" s="60"/>
-      <c r="G30" s="60"/>
-      <c r="H30" s="60"/>
-      <c r="I30" s="60"/>
-      <c r="J30" s="60"/>
-      <c r="K30" s="60"/>
-      <c r="L30" s="60"/>
-      <c r="M30" s="60"/>
-      <c r="N30" s="60"/>
-      <c r="O30" s="60"/>
-      <c r="P30" s="60"/>
-      <c r="Q30" s="60"/>
-      <c r="R30" s="60"/>
-      <c r="S30" s="60"/>
-      <c r="T30" s="60"/>
-      <c r="U30" s="60"/>
-      <c r="V30" s="60"/>
-      <c r="W30" s="60"/>
-      <c r="X30" s="60"/>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A30" s="24"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="24"/>
+      <c r="J30" s="24"/>
+      <c r="K30" s="24"/>
+      <c r="L30" s="24"/>
+      <c r="M30" s="24"/>
+      <c r="N30" s="24"/>
+      <c r="O30" s="24"/>
+      <c r="P30" s="24"/>
+      <c r="Q30" s="24"/>
+      <c r="R30" s="24"/>
+      <c r="S30" s="24"/>
+      <c r="T30" s="24"/>
+      <c r="U30" s="24"/>
+      <c r="V30" s="24"/>
+      <c r="W30" s="24"/>
+      <c r="X30" s="24"/>
     </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A31" s="60"/>
-      <c r="B31" s="60"/>
-      <c r="C31" s="60"/>
-      <c r="D31" s="60"/>
-      <c r="E31" s="60"/>
-      <c r="F31" s="60"/>
-      <c r="G31" s="60"/>
-      <c r="H31" s="60"/>
-      <c r="I31" s="60"/>
-      <c r="J31" s="60"/>
-      <c r="K31" s="60"/>
-      <c r="L31" s="60"/>
-      <c r="M31" s="60"/>
-      <c r="N31" s="60"/>
-      <c r="O31" s="60"/>
-      <c r="P31" s="60"/>
-      <c r="Q31" s="60"/>
-      <c r="R31" s="60"/>
-      <c r="S31" s="60"/>
-      <c r="T31" s="60"/>
-      <c r="U31" s="60"/>
-      <c r="V31" s="60"/>
-      <c r="W31" s="60"/>
-      <c r="X31" s="60"/>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A31" s="24"/>
+      <c r="B31" s="24"/>
+      <c r="C31" s="24"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="24"/>
+      <c r="J31" s="24"/>
+      <c r="K31" s="24"/>
+      <c r="L31" s="24"/>
+      <c r="M31" s="24"/>
+      <c r="N31" s="24"/>
+      <c r="O31" s="24"/>
+      <c r="P31" s="24"/>
+      <c r="Q31" s="24"/>
+      <c r="R31" s="24"/>
+      <c r="S31" s="24"/>
+      <c r="T31" s="24"/>
+      <c r="U31" s="24"/>
+      <c r="V31" s="24"/>
+      <c r="W31" s="24"/>
+      <c r="X31" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>